<commit_message>
Updated data type of analog outputs
</commit_message>
<xml_diff>
--- a/zero-data/io_lists/ZERO mocked IO-List.xlsx
+++ b/zero-data/io_lists/ZERO mocked IO-List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Repos\Git\zero\zero-data\io_lists\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B5B93BC-BED7-4CB7-88A5-ADCEC14CA31D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{494725B5-9FCC-4DB1-B2FD-6C30BA26320A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3270,20 +3270,24 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" textRotation="90"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" textRotation="90"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" textRotation="90"/>
     </xf>
@@ -3292,7 +3296,6 @@
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="11" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -3311,33 +3314,24 @@
       <alignment horizontal="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -3348,7 +3342,13 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4505,197 +4505,197 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:74" s="16" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="131" t="s">
+      <c r="A1" s="111" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="111" t="s">
+      <c r="B1" s="112" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="111" t="s">
+      <c r="C1" s="112" t="s">
         <v>49</v>
       </c>
-      <c r="D1" s="111" t="s">
+      <c r="D1" s="112" t="s">
         <v>50</v>
       </c>
-      <c r="E1" s="111" t="s">
+      <c r="E1" s="112" t="s">
         <v>51</v>
       </c>
-      <c r="F1" s="111" t="s">
+      <c r="F1" s="112" t="s">
         <v>52</v>
       </c>
-      <c r="G1" s="111" t="s">
+      <c r="G1" s="112" t="s">
         <v>53</v>
       </c>
-      <c r="H1" s="115" t="s">
+      <c r="H1" s="116" t="s">
         <v>54</v>
       </c>
-      <c r="I1" s="127" t="s">
+      <c r="I1" s="117" t="s">
         <v>55</v>
       </c>
-      <c r="J1" s="120" t="s">
+      <c r="J1" s="118" t="s">
         <v>56</v>
       </c>
-      <c r="K1" s="128" t="s">
+      <c r="K1" s="113" t="s">
         <v>3</v>
       </c>
-      <c r="L1" s="129" t="s">
+      <c r="L1" s="114" t="s">
         <v>64</v>
       </c>
-      <c r="M1" s="130"/>
-      <c r="N1" s="111" t="s">
+      <c r="M1" s="115"/>
+      <c r="N1" s="112" t="s">
         <v>57</v>
       </c>
-      <c r="O1" s="111" t="s">
+      <c r="O1" s="112" t="s">
         <v>58</v>
       </c>
-      <c r="P1" s="111" t="s">
+      <c r="P1" s="112" t="s">
         <v>59</v>
       </c>
-      <c r="Q1" s="111" t="s">
+      <c r="Q1" s="112" t="s">
         <v>60</v>
       </c>
-      <c r="R1" s="111" t="s">
+      <c r="R1" s="112" t="s">
         <v>61</v>
       </c>
-      <c r="S1" s="111" t="s">
+      <c r="S1" s="112" t="s">
         <v>62</v>
       </c>
-      <c r="T1" s="118" t="s">
+      <c r="T1" s="120" t="s">
         <v>63</v>
       </c>
-      <c r="U1" s="118"/>
-      <c r="V1" s="118"/>
-      <c r="W1" s="121" t="s">
+      <c r="U1" s="120"/>
+      <c r="V1" s="120"/>
+      <c r="W1" s="122" t="s">
         <v>438</v>
       </c>
-      <c r="X1" s="122"/>
-      <c r="Y1" s="122"/>
-      <c r="Z1" s="123"/>
-      <c r="AA1" s="119" t="s">
+      <c r="X1" s="123"/>
+      <c r="Y1" s="123"/>
+      <c r="Z1" s="124"/>
+      <c r="AA1" s="121" t="s">
         <v>27</v>
       </c>
-      <c r="AB1" s="119"/>
-      <c r="AC1" s="119"/>
-      <c r="AD1" s="119"/>
-      <c r="AE1" s="119"/>
-      <c r="AF1" s="119"/>
-      <c r="AG1" s="119"/>
-      <c r="AH1" s="119"/>
-      <c r="AI1" s="124" t="s">
+      <c r="AB1" s="121"/>
+      <c r="AC1" s="121"/>
+      <c r="AD1" s="121"/>
+      <c r="AE1" s="121"/>
+      <c r="AF1" s="121"/>
+      <c r="AG1" s="121"/>
+      <c r="AH1" s="121"/>
+      <c r="AI1" s="125" t="s">
         <v>65</v>
       </c>
-      <c r="AJ1" s="124"/>
-      <c r="AK1" s="120" t="s">
+      <c r="AJ1" s="125"/>
+      <c r="AK1" s="118" t="s">
         <v>66</v>
       </c>
-      <c r="AL1" s="120" t="s">
+      <c r="AL1" s="118" t="s">
         <v>67</v>
       </c>
-      <c r="AM1" s="117" t="s">
+      <c r="AM1" s="119" t="s">
         <v>68</v>
       </c>
-      <c r="AN1" s="126" t="s">
+      <c r="AN1" s="127" t="s">
         <v>69</v>
       </c>
-      <c r="AO1" s="126"/>
-      <c r="AP1" s="126"/>
-      <c r="AQ1" s="126"/>
-      <c r="AR1" s="126"/>
-      <c r="AS1" s="111" t="s">
+      <c r="AO1" s="127"/>
+      <c r="AP1" s="127"/>
+      <c r="AQ1" s="127"/>
+      <c r="AR1" s="127"/>
+      <c r="AS1" s="112" t="s">
         <v>70</v>
       </c>
-      <c r="AT1" s="111" t="s">
+      <c r="AT1" s="112" t="s">
         <v>71</v>
       </c>
-      <c r="AU1" s="111" t="s">
+      <c r="AU1" s="112" t="s">
         <v>72</v>
       </c>
-      <c r="AV1" s="111" t="s">
+      <c r="AV1" s="112" t="s">
         <v>73</v>
       </c>
-      <c r="AW1" s="125" t="s">
+      <c r="AW1" s="126" t="s">
         <v>74</v>
       </c>
-      <c r="AX1" s="114" t="s">
+      <c r="AX1" s="130" t="s">
         <v>75</v>
       </c>
-      <c r="AY1" s="115" t="s">
+      <c r="AY1" s="116" t="s">
         <v>76</v>
       </c>
-      <c r="AZ1" s="115" t="s">
+      <c r="AZ1" s="116" t="s">
         <v>77</v>
       </c>
-      <c r="BA1" s="115" t="s">
+      <c r="BA1" s="116" t="s">
         <v>78</v>
       </c>
-      <c r="BB1" s="115" t="s">
+      <c r="BB1" s="116" t="s">
         <v>79</v>
       </c>
-      <c r="BC1" s="113" t="s">
+      <c r="BC1" s="129" t="s">
         <v>80</v>
       </c>
-      <c r="BD1" s="113"/>
-      <c r="BE1" s="113"/>
-      <c r="BF1" s="113" t="s">
+      <c r="BD1" s="129"/>
+      <c r="BE1" s="129"/>
+      <c r="BF1" s="129" t="s">
         <v>81</v>
       </c>
-      <c r="BG1" s="113"/>
-      <c r="BH1" s="113"/>
-      <c r="BI1" s="113" t="s">
+      <c r="BG1" s="129"/>
+      <c r="BH1" s="129"/>
+      <c r="BI1" s="129" t="s">
         <v>82</v>
       </c>
-      <c r="BJ1" s="113"/>
-      <c r="BK1" s="113"/>
-      <c r="BL1" s="113" t="s">
+      <c r="BJ1" s="129"/>
+      <c r="BK1" s="129"/>
+      <c r="BL1" s="129" t="s">
         <v>83</v>
       </c>
-      <c r="BM1" s="113"/>
-      <c r="BN1" s="113"/>
-      <c r="BO1" s="113" t="s">
+      <c r="BM1" s="129"/>
+      <c r="BN1" s="129"/>
+      <c r="BO1" s="129" t="s">
         <v>84</v>
       </c>
-      <c r="BP1" s="113"/>
-      <c r="BQ1" s="113"/>
-      <c r="BR1" s="117" t="s">
+      <c r="BP1" s="129"/>
+      <c r="BQ1" s="129"/>
+      <c r="BR1" s="119" t="s">
         <v>85</v>
       </c>
-      <c r="BS1" s="115" t="s">
+      <c r="BS1" s="116" t="s">
         <v>86</v>
       </c>
-      <c r="BT1" s="116" t="s">
+      <c r="BT1" s="131" t="s">
         <v>87</v>
       </c>
-      <c r="BU1" s="112" t="s">
+      <c r="BU1" s="128" t="s">
         <v>88</v>
       </c>
-      <c r="BV1" s="112" t="s">
+      <c r="BV1" s="128" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:74" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="131"/>
-      <c r="B2" s="111"/>
-      <c r="C2" s="111"/>
-      <c r="D2" s="111"/>
-      <c r="E2" s="111"/>
-      <c r="F2" s="111"/>
-      <c r="G2" s="111"/>
-      <c r="H2" s="115"/>
-      <c r="I2" s="127"/>
-      <c r="J2" s="120"/>
-      <c r="K2" s="128"/>
+      <c r="A2" s="111"/>
+      <c r="B2" s="112"/>
+      <c r="C2" s="112"/>
+      <c r="D2" s="112"/>
+      <c r="E2" s="112"/>
+      <c r="F2" s="112"/>
+      <c r="G2" s="112"/>
+      <c r="H2" s="116"/>
+      <c r="I2" s="117"/>
+      <c r="J2" s="118"/>
+      <c r="K2" s="113"/>
       <c r="L2" s="97" t="s">
         <v>93</v>
       </c>
       <c r="M2" s="97" t="s">
         <v>94</v>
       </c>
-      <c r="N2" s="111"/>
-      <c r="O2" s="111"/>
-      <c r="P2" s="111"/>
-      <c r="Q2" s="111"/>
-      <c r="R2" s="111"/>
-      <c r="S2" s="111"/>
+      <c r="N2" s="112"/>
+      <c r="O2" s="112"/>
+      <c r="P2" s="112"/>
+      <c r="Q2" s="112"/>
+      <c r="R2" s="112"/>
+      <c r="S2" s="112"/>
       <c r="T2" s="17" t="s">
         <v>90</v>
       </c>
@@ -4747,9 +4747,9 @@
       <c r="AJ2" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="AK2" s="120"/>
-      <c r="AL2" s="120"/>
-      <c r="AM2" s="117"/>
+      <c r="AK2" s="118"/>
+      <c r="AL2" s="118"/>
+      <c r="AM2" s="119"/>
       <c r="AN2" s="18" t="s">
         <v>103</v>
       </c>
@@ -4765,16 +4765,16 @@
       <c r="AR2" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="AS2" s="111"/>
-      <c r="AT2" s="111"/>
-      <c r="AU2" s="111"/>
-      <c r="AV2" s="111"/>
-      <c r="AW2" s="125"/>
-      <c r="AX2" s="114"/>
-      <c r="AY2" s="115"/>
-      <c r="AZ2" s="115"/>
-      <c r="BA2" s="115"/>
-      <c r="BB2" s="115"/>
+      <c r="AS2" s="112"/>
+      <c r="AT2" s="112"/>
+      <c r="AU2" s="112"/>
+      <c r="AV2" s="112"/>
+      <c r="AW2" s="126"/>
+      <c r="AX2" s="130"/>
+      <c r="AY2" s="116"/>
+      <c r="AZ2" s="116"/>
+      <c r="BA2" s="116"/>
+      <c r="BB2" s="116"/>
       <c r="BC2" s="21" t="s">
         <v>56</v>
       </c>
@@ -4820,11 +4820,11 @@
       <c r="BQ2" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="BR2" s="117"/>
-      <c r="BS2" s="115"/>
-      <c r="BT2" s="116"/>
-      <c r="BU2" s="112"/>
-      <c r="BV2" s="112"/>
+      <c r="BR2" s="119"/>
+      <c r="BS2" s="116"/>
+      <c r="BT2" s="131"/>
+      <c r="BU2" s="128"/>
+      <c r="BV2" s="128"/>
     </row>
     <row r="3" spans="1:74" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="50" t="s">
@@ -7222,7 +7222,7 @@
         <v>376</v>
       </c>
       <c r="C30" s="54" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="D30" s="7" t="s">
         <v>521</v>
@@ -7257,7 +7257,7 @@
         <v>376</v>
       </c>
       <c r="C31" s="54" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>521</v>
@@ -7292,7 +7292,7 @@
         <v>376</v>
       </c>
       <c r="C32" s="54" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="D32" s="7" t="s">
         <v>521</v>
@@ -7747,7 +7747,7 @@
         <v>376</v>
       </c>
       <c r="C45" s="54" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="D45" s="7" t="s">
         <v>557</v>
@@ -7782,7 +7782,7 @@
         <v>376</v>
       </c>
       <c r="C46" s="54" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="D46" s="7" t="s">
         <v>557</v>
@@ -7817,7 +7817,7 @@
         <v>376</v>
       </c>
       <c r="C47" s="54" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="D47" s="7" t="s">
         <v>557</v>
@@ -63086,36 +63086,6 @@
     <filterColumn colId="67" showButton="0"/>
   </autoFilter>
   <mergeCells count="46">
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="K1:K2"/>
-    <mergeCell ref="N1:N2"/>
-    <mergeCell ref="O1:O2"/>
-    <mergeCell ref="P1:P2"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="J1:J2"/>
-    <mergeCell ref="S1:S2"/>
-    <mergeCell ref="BR1:BR2"/>
-    <mergeCell ref="T1:V1"/>
-    <mergeCell ref="AA1:AH1"/>
-    <mergeCell ref="AM1:AM2"/>
-    <mergeCell ref="AK1:AK2"/>
-    <mergeCell ref="AL1:AL2"/>
-    <mergeCell ref="W1:Z1"/>
-    <mergeCell ref="AI1:AJ1"/>
-    <mergeCell ref="AS1:AS2"/>
-    <mergeCell ref="AT1:AT2"/>
-    <mergeCell ref="AU1:AU2"/>
-    <mergeCell ref="AV1:AV2"/>
-    <mergeCell ref="AW1:AW2"/>
-    <mergeCell ref="AN1:AR1"/>
     <mergeCell ref="Q1:Q2"/>
     <mergeCell ref="BV1:BV2"/>
     <mergeCell ref="BC1:BE1"/>
@@ -63132,6 +63102,36 @@
     <mergeCell ref="BT1:BT2"/>
     <mergeCell ref="BU1:BU2"/>
     <mergeCell ref="R1:R2"/>
+    <mergeCell ref="S1:S2"/>
+    <mergeCell ref="BR1:BR2"/>
+    <mergeCell ref="T1:V1"/>
+    <mergeCell ref="AA1:AH1"/>
+    <mergeCell ref="AM1:AM2"/>
+    <mergeCell ref="AK1:AK2"/>
+    <mergeCell ref="AL1:AL2"/>
+    <mergeCell ref="W1:Z1"/>
+    <mergeCell ref="AI1:AJ1"/>
+    <mergeCell ref="AS1:AS2"/>
+    <mergeCell ref="AT1:AT2"/>
+    <mergeCell ref="AU1:AU2"/>
+    <mergeCell ref="AV1:AV2"/>
+    <mergeCell ref="AW1:AW2"/>
+    <mergeCell ref="AN1:AR1"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="J1:J2"/>
+    <mergeCell ref="K1:K2"/>
+    <mergeCell ref="N1:N2"/>
+    <mergeCell ref="O1:O2"/>
+    <mergeCell ref="P1:P2"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <dataValidations count="1">
@@ -63226,10 +63226,10 @@
       <c r="A4" s="25" t="s">
         <v>153</v>
       </c>
-      <c r="B4" s="140" t="s">
+      <c r="B4" s="132" t="s">
         <v>154</v>
       </c>
-      <c r="C4" s="140"/>
+      <c r="C4" s="132"/>
       <c r="D4" s="26" t="s">
         <v>59</v>
       </c>
@@ -63238,13 +63238,13 @@
       </c>
     </row>
     <row r="5" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="132" t="s">
+      <c r="A5" s="133" t="s">
         <v>156</v>
       </c>
-      <c r="B5" s="132" t="s">
+      <c r="B5" s="133" t="s">
         <v>157</v>
       </c>
-      <c r="C5" s="132"/>
+      <c r="C5" s="133"/>
       <c r="D5" s="28" t="s">
         <v>158</v>
       </c>
@@ -63253,16 +63253,16 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="132"/>
-      <c r="B6" s="132"/>
-      <c r="C6" s="132"/>
+      <c r="A6" s="133"/>
+      <c r="B6" s="133"/>
+      <c r="C6" s="133"/>
       <c r="D6" s="28"/>
       <c r="E6" s="30"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="132"/>
-      <c r="B7" s="132"/>
-      <c r="C7" s="132"/>
+      <c r="A7" s="133"/>
+      <c r="B7" s="133"/>
+      <c r="C7" s="133"/>
       <c r="D7" s="28" t="s">
         <v>160</v>
       </c>
@@ -63271,9 +63271,9 @@
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="132"/>
-      <c r="B8" s="132"/>
-      <c r="C8" s="132"/>
+      <c r="A8" s="133"/>
+      <c r="B8" s="133"/>
+      <c r="C8" s="133"/>
       <c r="D8" s="28" t="s">
         <v>162</v>
       </c>
@@ -63282,9 +63282,9 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="132"/>
-      <c r="B9" s="132"/>
-      <c r="C9" s="132"/>
+      <c r="A9" s="133"/>
+      <c r="B9" s="133"/>
+      <c r="C9" s="133"/>
       <c r="D9" s="28" t="s">
         <v>163</v>
       </c>
@@ -63293,9 +63293,9 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="132"/>
-      <c r="B10" s="132"/>
-      <c r="C10" s="132"/>
+      <c r="A10" s="133"/>
+      <c r="B10" s="133"/>
+      <c r="C10" s="133"/>
       <c r="D10" s="28" t="s">
         <v>164</v>
       </c>
@@ -63304,9 +63304,9 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="132"/>
-      <c r="B11" s="132"/>
-      <c r="C11" s="132"/>
+      <c r="A11" s="133"/>
+      <c r="B11" s="133"/>
+      <c r="C11" s="133"/>
       <c r="D11" s="31" t="s">
         <v>165</v>
       </c>
@@ -63318,7 +63318,7 @@
       <c r="A12" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B12" s="132" t="s">
+      <c r="B12" s="133" t="s">
         <v>166</v>
       </c>
       <c r="C12" s="31" t="s">
@@ -63335,7 +63335,7 @@
       <c r="A13" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B13" s="132"/>
+      <c r="B13" s="133"/>
       <c r="C13" s="31" t="s">
         <v>104</v>
       </c>
@@ -63350,7 +63350,7 @@
       <c r="A14" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B14" s="132"/>
+      <c r="B14" s="133"/>
       <c r="C14" s="31" t="s">
         <v>105</v>
       </c>
@@ -63365,7 +63365,7 @@
       <c r="A15" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B15" s="132"/>
+      <c r="B15" s="133"/>
       <c r="C15" s="31" t="s">
         <v>106</v>
       </c>
@@ -63380,7 +63380,7 @@
       <c r="A16" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B16" s="132"/>
+      <c r="B16" s="133"/>
       <c r="C16" s="31" t="s">
         <v>107</v>
       </c>
@@ -63395,10 +63395,10 @@
       <c r="A17" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B17" s="132" t="s">
+      <c r="B17" s="133" t="s">
         <v>68</v>
       </c>
-      <c r="C17" s="132"/>
+      <c r="C17" s="133"/>
       <c r="D17" s="31" t="s">
         <v>177</v>
       </c>
@@ -63410,10 +63410,10 @@
       <c r="A18" s="32" t="s">
         <v>179</v>
       </c>
-      <c r="B18" s="132" t="s">
+      <c r="B18" s="133" t="s">
         <v>3</v>
       </c>
-      <c r="C18" s="132"/>
+      <c r="C18" s="133"/>
       <c r="D18" s="31" t="s">
         <v>180</v>
       </c>
@@ -63425,10 +63425,10 @@
       <c r="A19" s="32" t="s">
         <v>179</v>
       </c>
-      <c r="B19" s="132" t="s">
+      <c r="B19" s="133" t="s">
         <v>182</v>
       </c>
-      <c r="C19" s="132"/>
+      <c r="C19" s="133"/>
       <c r="D19" s="31" t="s">
         <v>183</v>
       </c>
@@ -63440,10 +63440,10 @@
       <c r="A20" s="32" t="s">
         <v>179</v>
       </c>
-      <c r="B20" s="132" t="s">
+      <c r="B20" s="133" t="s">
         <v>185</v>
       </c>
-      <c r="C20" s="132"/>
+      <c r="C20" s="133"/>
       <c r="D20" s="31" t="s">
         <v>186</v>
       </c>
@@ -63455,10 +63455,10 @@
       <c r="A21" s="32" t="s">
         <v>179</v>
       </c>
-      <c r="B21" s="132" t="s">
+      <c r="B21" s="133" t="s">
         <v>188</v>
       </c>
-      <c r="C21" s="132"/>
+      <c r="C21" s="133"/>
       <c r="D21" s="31" t="s">
         <v>189</v>
       </c>
@@ -63470,10 +63470,10 @@
       <c r="A22" s="32" t="s">
         <v>179</v>
       </c>
-      <c r="B22" s="132" t="s">
+      <c r="B22" s="133" t="s">
         <v>191</v>
       </c>
-      <c r="C22" s="132"/>
+      <c r="C22" s="133"/>
       <c r="D22" s="31" t="s">
         <v>192</v>
       </c>
@@ -63482,13 +63482,13 @@
       </c>
     </row>
     <row r="23" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="132" t="s">
+      <c r="A23" s="133" t="s">
         <v>156</v>
       </c>
-      <c r="B23" s="132" t="s">
+      <c r="B23" s="133" t="s">
         <v>96</v>
       </c>
-      <c r="C23" s="132"/>
+      <c r="C23" s="133"/>
       <c r="D23" s="28" t="s">
         <v>194</v>
       </c>
@@ -63497,9 +63497,9 @@
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="132"/>
-      <c r="B24" s="132"/>
-      <c r="C24" s="132"/>
+      <c r="A24" s="133"/>
+      <c r="B24" s="133"/>
+      <c r="C24" s="133"/>
       <c r="D24" s="28" t="s">
         <v>196</v>
       </c>
@@ -63508,9 +63508,9 @@
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="132"/>
-      <c r="B25" s="132"/>
-      <c r="C25" s="132"/>
+      <c r="A25" s="133"/>
+      <c r="B25" s="133"/>
+      <c r="C25" s="133"/>
       <c r="D25" s="28" t="s">
         <v>198</v>
       </c>
@@ -63519,9 +63519,9 @@
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="132"/>
-      <c r="B26" s="132"/>
-      <c r="C26" s="132"/>
+      <c r="A26" s="133"/>
+      <c r="B26" s="133"/>
+      <c r="C26" s="133"/>
       <c r="D26" s="28" t="s">
         <v>199</v>
       </c>
@@ -63530,9 +63530,9 @@
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="132"/>
-      <c r="B27" s="132"/>
-      <c r="C27" s="132"/>
+      <c r="A27" s="133"/>
+      <c r="B27" s="133"/>
+      <c r="C27" s="133"/>
       <c r="D27" s="28" t="s">
         <v>200</v>
       </c>
@@ -63541,9 +63541,9 @@
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="132"/>
-      <c r="B28" s="132"/>
-      <c r="C28" s="132"/>
+      <c r="A28" s="133"/>
+      <c r="B28" s="133"/>
+      <c r="C28" s="133"/>
       <c r="D28" s="28" t="s">
         <v>201</v>
       </c>
@@ -63552,9 +63552,9 @@
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="132"/>
-      <c r="B29" s="132"/>
-      <c r="C29" s="132"/>
+      <c r="A29" s="133"/>
+      <c r="B29" s="133"/>
+      <c r="C29" s="133"/>
       <c r="D29" s="28" t="s">
         <v>202</v>
       </c>
@@ -63563,9 +63563,9 @@
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="132"/>
-      <c r="B30" s="132"/>
-      <c r="C30" s="132"/>
+      <c r="A30" s="133"/>
+      <c r="B30" s="133"/>
+      <c r="C30" s="133"/>
       <c r="D30" s="28" t="s">
         <v>203</v>
       </c>
@@ -63574,9 +63574,9 @@
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="132"/>
-      <c r="B31" s="132"/>
-      <c r="C31" s="132"/>
+      <c r="A31" s="133"/>
+      <c r="B31" s="133"/>
+      <c r="C31" s="133"/>
       <c r="D31" s="28" t="s">
         <v>204</v>
       </c>
@@ -63585,9 +63585,9 @@
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="132"/>
-      <c r="B32" s="132"/>
-      <c r="C32" s="132"/>
+      <c r="A32" s="133"/>
+      <c r="B32" s="133"/>
+      <c r="C32" s="133"/>
       <c r="D32" s="28" t="s">
         <v>205</v>
       </c>
@@ -63596,9 +63596,9 @@
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="132"/>
-      <c r="B33" s="132"/>
-      <c r="C33" s="132"/>
+      <c r="A33" s="133"/>
+      <c r="B33" s="133"/>
+      <c r="C33" s="133"/>
       <c r="D33" s="28" t="s">
         <v>206</v>
       </c>
@@ -63607,16 +63607,16 @@
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="132"/>
-      <c r="B34" s="132"/>
-      <c r="C34" s="132"/>
+      <c r="A34" s="133"/>
+      <c r="B34" s="133"/>
+      <c r="C34" s="133"/>
       <c r="D34" s="28"/>
       <c r="E34" s="30"/>
     </row>
     <row r="35" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A35" s="132"/>
-      <c r="B35" s="132"/>
-      <c r="C35" s="132"/>
+      <c r="A35" s="133"/>
+      <c r="B35" s="133"/>
+      <c r="C35" s="133"/>
       <c r="D35" s="28" t="s">
         <v>208</v>
       </c>
@@ -63625,9 +63625,9 @@
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="132"/>
-      <c r="B36" s="132"/>
-      <c r="C36" s="132"/>
+      <c r="A36" s="133"/>
+      <c r="B36" s="133"/>
+      <c r="C36" s="133"/>
       <c r="D36" s="31" t="s">
         <v>210</v>
       </c>
@@ -63639,10 +63639,10 @@
       <c r="A37" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B37" s="133" t="s">
+      <c r="B37" s="134" t="s">
         <v>70</v>
       </c>
-      <c r="C37" s="133"/>
+      <c r="C37" s="134"/>
       <c r="D37" s="31" t="s">
         <v>212</v>
       </c>
@@ -63654,10 +63654,10 @@
       <c r="A38" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B38" s="132" t="s">
+      <c r="B38" s="133" t="s">
         <v>48</v>
       </c>
-      <c r="C38" s="132"/>
+      <c r="C38" s="133"/>
       <c r="D38" s="31" t="s">
         <v>214</v>
       </c>
@@ -63669,10 +63669,10 @@
       <c r="A39" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B39" s="132" t="s">
+      <c r="B39" s="133" t="s">
         <v>59</v>
       </c>
-      <c r="C39" s="132"/>
+      <c r="C39" s="133"/>
       <c r="D39" s="31" t="s">
         <v>216</v>
       </c>
@@ -63681,13 +63681,13 @@
       </c>
     </row>
     <row r="40" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="132" t="s">
+      <c r="A40" s="133" t="s">
         <v>156</v>
       </c>
-      <c r="B40" s="132" t="s">
+      <c r="B40" s="133" t="s">
         <v>50</v>
       </c>
-      <c r="C40" s="132"/>
+      <c r="C40" s="133"/>
       <c r="D40" s="28" t="s">
         <v>218</v>
       </c>
@@ -63696,9 +63696,9 @@
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="132"/>
-      <c r="B41" s="132"/>
-      <c r="C41" s="132"/>
+      <c r="A41" s="133"/>
+      <c r="B41" s="133"/>
+      <c r="C41" s="133"/>
       <c r="D41" s="28" t="s">
         <v>220</v>
       </c>
@@ -63707,9 +63707,9 @@
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="132"/>
-      <c r="B42" s="132"/>
-      <c r="C42" s="132"/>
+      <c r="A42" s="133"/>
+      <c r="B42" s="133"/>
+      <c r="C42" s="133"/>
       <c r="D42" s="28" t="s">
         <v>222</v>
       </c>
@@ -63718,9 +63718,9 @@
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="132"/>
-      <c r="B43" s="132"/>
-      <c r="C43" s="132"/>
+      <c r="A43" s="133"/>
+      <c r="B43" s="133"/>
+      <c r="C43" s="133"/>
       <c r="D43" s="28" t="s">
         <v>224</v>
       </c>
@@ -63729,9 +63729,9 @@
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="132"/>
-      <c r="B44" s="132"/>
-      <c r="C44" s="132"/>
+      <c r="A44" s="133"/>
+      <c r="B44" s="133"/>
+      <c r="C44" s="133"/>
       <c r="D44" s="28" t="s">
         <v>226</v>
       </c>
@@ -63743,10 +63743,10 @@
       <c r="A45" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B45" s="132" t="s">
+      <c r="B45" s="133" t="s">
         <v>78</v>
       </c>
-      <c r="C45" s="132"/>
+      <c r="C45" s="133"/>
       <c r="D45" s="27" t="s">
         <v>227</v>
       </c>
@@ -63803,7 +63803,7 @@
       <c r="A49" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B49" s="137" t="s">
+      <c r="B49" s="135" t="s">
         <v>237</v>
       </c>
       <c r="C49" s="31" t="s">
@@ -63817,11 +63817,11 @@
       </c>
     </row>
     <row r="50" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="132" t="s">
+      <c r="A50" s="133" t="s">
         <v>156</v>
       </c>
-      <c r="B50" s="137"/>
-      <c r="C50" s="138" t="s">
+      <c r="B50" s="135"/>
+      <c r="C50" s="136" t="s">
         <v>108</v>
       </c>
       <c r="D50" s="40" t="s">
@@ -63832,9 +63832,9 @@
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" s="132"/>
-      <c r="B51" s="137"/>
-      <c r="C51" s="138"/>
+      <c r="A51" s="133"/>
+      <c r="B51" s="135"/>
+      <c r="C51" s="136"/>
       <c r="D51" s="30" t="s">
         <v>242</v>
       </c>
@@ -63843,9 +63843,9 @@
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="132"/>
-      <c r="B52" s="137"/>
-      <c r="C52" s="138"/>
+      <c r="A52" s="133"/>
+      <c r="B52" s="135"/>
+      <c r="C52" s="136"/>
       <c r="D52" s="30" t="s">
         <v>244</v>
       </c>
@@ -63854,9 +63854,9 @@
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="132"/>
-      <c r="B53" s="137"/>
-      <c r="C53" s="138"/>
+      <c r="A53" s="133"/>
+      <c r="B53" s="135"/>
+      <c r="C53" s="136"/>
       <c r="D53" s="30" t="s">
         <v>246</v>
       </c>
@@ -63865,16 +63865,16 @@
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="132"/>
-      <c r="B54" s="137"/>
-      <c r="C54" s="138"/>
+      <c r="A54" s="133"/>
+      <c r="B54" s="135"/>
+      <c r="C54" s="136"/>
       <c r="D54" s="28"/>
       <c r="E54" s="30"/>
     </row>
     <row r="55" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A55" s="132"/>
-      <c r="B55" s="137"/>
-      <c r="C55" s="138"/>
+      <c r="A55" s="133"/>
+      <c r="B55" s="135"/>
+      <c r="C55" s="136"/>
       <c r="D55" s="31" t="s">
         <v>248</v>
       </c>
@@ -63883,11 +63883,11 @@
       </c>
     </row>
     <row r="56" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="132" t="s">
+      <c r="A56" s="133" t="s">
         <v>156</v>
       </c>
-      <c r="B56" s="137"/>
-      <c r="C56" s="139" t="s">
+      <c r="B56" s="135"/>
+      <c r="C56" s="137" t="s">
         <v>109</v>
       </c>
       <c r="D56" s="28" t="s">
@@ -63898,9 +63898,9 @@
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="132"/>
-      <c r="B57" s="137"/>
-      <c r="C57" s="139"/>
+      <c r="A57" s="133"/>
+      <c r="B57" s="135"/>
+      <c r="C57" s="137"/>
       <c r="D57" s="28" t="s">
         <v>252</v>
       </c>
@@ -63909,9 +63909,9 @@
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" s="132"/>
-      <c r="B58" s="137"/>
-      <c r="C58" s="139"/>
+      <c r="A58" s="133"/>
+      <c r="B58" s="135"/>
+      <c r="C58" s="137"/>
       <c r="D58" s="31" t="s">
         <v>254</v>
       </c>
@@ -63923,10 +63923,10 @@
       <c r="A59" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B59" s="132" t="s">
+      <c r="B59" s="133" t="s">
         <v>76</v>
       </c>
-      <c r="C59" s="132"/>
+      <c r="C59" s="133"/>
       <c r="D59" s="31" t="s">
         <v>256</v>
       </c>
@@ -63938,7 +63938,7 @@
       <c r="A60" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B60" s="136" t="s">
+      <c r="B60" s="138" t="s">
         <v>82</v>
       </c>
       <c r="C60" s="31" t="s">
@@ -63952,11 +63952,11 @@
       </c>
     </row>
     <row r="61" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="132" t="s">
+      <c r="A61" s="133" t="s">
         <v>156</v>
       </c>
-      <c r="B61" s="136"/>
-      <c r="C61" s="132" t="s">
+      <c r="B61" s="138"/>
+      <c r="C61" s="133" t="s">
         <v>108</v>
       </c>
       <c r="D61" s="40" t="s">
@@ -63967,9 +63967,9 @@
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" s="132"/>
-      <c r="B62" s="132"/>
-      <c r="C62" s="132"/>
+      <c r="A62" s="133"/>
+      <c r="B62" s="133"/>
+      <c r="C62" s="133"/>
       <c r="D62" s="30" t="s">
         <v>242</v>
       </c>
@@ -63978,9 +63978,9 @@
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A63" s="132"/>
-      <c r="B63" s="132"/>
-      <c r="C63" s="132"/>
+      <c r="A63" s="133"/>
+      <c r="B63" s="133"/>
+      <c r="C63" s="133"/>
       <c r="D63" s="30" t="s">
         <v>244</v>
       </c>
@@ -63989,9 +63989,9 @@
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64" s="132"/>
-      <c r="B64" s="132"/>
-      <c r="C64" s="132"/>
+      <c r="A64" s="133"/>
+      <c r="B64" s="133"/>
+      <c r="C64" s="133"/>
       <c r="D64" s="30" t="s">
         <v>246</v>
       </c>
@@ -64000,16 +64000,16 @@
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A65" s="132"/>
-      <c r="B65" s="132"/>
-      <c r="C65" s="132"/>
+      <c r="A65" s="133"/>
+      <c r="B65" s="133"/>
+      <c r="C65" s="133"/>
       <c r="D65" s="28"/>
       <c r="E65" s="30"/>
     </row>
     <row r="66" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A66" s="132"/>
-      <c r="B66" s="136"/>
-      <c r="C66" s="132"/>
+      <c r="A66" s="133"/>
+      <c r="B66" s="138"/>
+      <c r="C66" s="133"/>
       <c r="D66" s="31" t="s">
         <v>248</v>
       </c>
@@ -64018,11 +64018,11 @@
       </c>
     </row>
     <row r="67" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="132" t="s">
+      <c r="A67" s="133" t="s">
         <v>156</v>
       </c>
-      <c r="B67" s="136"/>
-      <c r="C67" s="132" t="s">
+      <c r="B67" s="138"/>
+      <c r="C67" s="133" t="s">
         <v>109</v>
       </c>
       <c r="D67" s="28" t="s">
@@ -64033,9 +64033,9 @@
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" s="132"/>
-      <c r="B68" s="132"/>
-      <c r="C68" s="132"/>
+      <c r="A68" s="133"/>
+      <c r="B68" s="133"/>
+      <c r="C68" s="133"/>
       <c r="D68" s="28" t="s">
         <v>252</v>
       </c>
@@ -64044,9 +64044,9 @@
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" s="132"/>
-      <c r="B69" s="136"/>
-      <c r="C69" s="132"/>
+      <c r="A69" s="133"/>
+      <c r="B69" s="138"/>
+      <c r="C69" s="133"/>
       <c r="D69" s="31" t="s">
         <v>254</v>
       </c>
@@ -64058,7 +64058,7 @@
       <c r="A70" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B70" s="136" t="s">
+      <c r="B70" s="138" t="s">
         <v>81</v>
       </c>
       <c r="C70" s="31" t="s">
@@ -64072,11 +64072,11 @@
       </c>
     </row>
     <row r="71" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="132" t="s">
+      <c r="A71" s="133" t="s">
         <v>156</v>
       </c>
-      <c r="B71" s="136"/>
-      <c r="C71" s="132" t="s">
+      <c r="B71" s="138"/>
+      <c r="C71" s="133" t="s">
         <v>108</v>
       </c>
       <c r="D71" s="40" t="s">
@@ -64087,9 +64087,9 @@
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A72" s="132"/>
-      <c r="B72" s="132"/>
-      <c r="C72" s="132"/>
+      <c r="A72" s="133"/>
+      <c r="B72" s="133"/>
+      <c r="C72" s="133"/>
       <c r="D72" s="30" t="s">
         <v>242</v>
       </c>
@@ -64098,9 +64098,9 @@
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A73" s="132"/>
-      <c r="B73" s="132"/>
-      <c r="C73" s="132"/>
+      <c r="A73" s="133"/>
+      <c r="B73" s="133"/>
+      <c r="C73" s="133"/>
       <c r="D73" s="30" t="s">
         <v>244</v>
       </c>
@@ -64109,9 +64109,9 @@
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A74" s="132"/>
-      <c r="B74" s="132"/>
-      <c r="C74" s="132"/>
+      <c r="A74" s="133"/>
+      <c r="B74" s="133"/>
+      <c r="C74" s="133"/>
       <c r="D74" s="30" t="s">
         <v>246</v>
       </c>
@@ -64120,16 +64120,16 @@
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A75" s="132"/>
-      <c r="B75" s="132"/>
-      <c r="C75" s="132"/>
+      <c r="A75" s="133"/>
+      <c r="B75" s="133"/>
+      <c r="C75" s="133"/>
       <c r="D75" s="28"/>
       <c r="E75" s="30"/>
     </row>
     <row r="76" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A76" s="132"/>
-      <c r="B76" s="136"/>
-      <c r="C76" s="132"/>
+      <c r="A76" s="133"/>
+      <c r="B76" s="138"/>
+      <c r="C76" s="133"/>
       <c r="D76" s="31" t="s">
         <v>248</v>
       </c>
@@ -64138,11 +64138,11 @@
       </c>
     </row>
     <row r="77" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="132" t="s">
+      <c r="A77" s="133" t="s">
         <v>156</v>
       </c>
-      <c r="B77" s="136"/>
-      <c r="C77" s="132" t="s">
+      <c r="B77" s="138"/>
+      <c r="C77" s="133" t="s">
         <v>109</v>
       </c>
       <c r="D77" s="28" t="s">
@@ -64153,9 +64153,9 @@
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A78" s="132"/>
-      <c r="B78" s="132"/>
-      <c r="C78" s="132"/>
+      <c r="A78" s="133"/>
+      <c r="B78" s="133"/>
+      <c r="C78" s="133"/>
       <c r="D78" s="28" t="s">
         <v>252</v>
       </c>
@@ -64164,9 +64164,9 @@
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A79" s="132"/>
-      <c r="B79" s="136"/>
-      <c r="C79" s="132"/>
+      <c r="A79" s="133"/>
+      <c r="B79" s="138"/>
+      <c r="C79" s="133"/>
       <c r="D79" s="31" t="s">
         <v>254</v>
       </c>
@@ -64175,13 +64175,13 @@
       </c>
     </row>
     <row r="80" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="132" t="s">
+      <c r="A80" s="133" t="s">
         <v>156</v>
       </c>
-      <c r="B80" s="132" t="s">
+      <c r="B80" s="133" t="s">
         <v>258</v>
       </c>
-      <c r="C80" s="132"/>
+      <c r="C80" s="133"/>
       <c r="D80" s="28" t="s">
         <v>259</v>
       </c>
@@ -64190,9 +64190,9 @@
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A81" s="132"/>
-      <c r="B81" s="132"/>
-      <c r="C81" s="132"/>
+      <c r="A81" s="133"/>
+      <c r="B81" s="133"/>
+      <c r="C81" s="133"/>
       <c r="D81" s="28" t="s">
         <v>261</v>
       </c>
@@ -64201,9 +64201,9 @@
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A82" s="132"/>
-      <c r="B82" s="132"/>
-      <c r="C82" s="132"/>
+      <c r="A82" s="133"/>
+      <c r="B82" s="133"/>
+      <c r="C82" s="133"/>
       <c r="D82" s="28" t="s">
         <v>263</v>
       </c>
@@ -64212,9 +64212,9 @@
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A83" s="132"/>
-      <c r="B83" s="132"/>
-      <c r="C83" s="132"/>
+      <c r="A83" s="133"/>
+      <c r="B83" s="133"/>
+      <c r="C83" s="133"/>
       <c r="D83" s="28" t="s">
         <v>265</v>
       </c>
@@ -64223,9 +64223,9 @@
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A84" s="132"/>
-      <c r="B84" s="132"/>
-      <c r="C84" s="132"/>
+      <c r="A84" s="133"/>
+      <c r="B84" s="133"/>
+      <c r="C84" s="133"/>
       <c r="D84" s="28" t="s">
         <v>267</v>
       </c>
@@ -64234,9 +64234,9 @@
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A85" s="132"/>
-      <c r="B85" s="132"/>
-      <c r="C85" s="132"/>
+      <c r="A85" s="133"/>
+      <c r="B85" s="133"/>
+      <c r="C85" s="133"/>
       <c r="D85" s="31" t="s">
         <v>269</v>
       </c>
@@ -64248,10 +64248,10 @@
       <c r="A86" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B86" s="132" t="s">
+      <c r="B86" s="133" t="s">
         <v>74</v>
       </c>
-      <c r="C86" s="132"/>
+      <c r="C86" s="133"/>
       <c r="D86" s="31" t="s">
         <v>271</v>
       </c>
@@ -64263,7 +64263,7 @@
       <c r="A87" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B87" s="136" t="s">
+      <c r="B87" s="138" t="s">
         <v>83</v>
       </c>
       <c r="C87" s="31" t="s">
@@ -64277,11 +64277,11 @@
       </c>
     </row>
     <row r="88" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="132" t="s">
+      <c r="A88" s="133" t="s">
         <v>156</v>
       </c>
-      <c r="B88" s="136"/>
-      <c r="C88" s="132" t="s">
+      <c r="B88" s="138"/>
+      <c r="C88" s="133" t="s">
         <v>108</v>
       </c>
       <c r="D88" s="40" t="s">
@@ -64292,9 +64292,9 @@
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A89" s="132"/>
-      <c r="B89" s="132"/>
-      <c r="C89" s="132"/>
+      <c r="A89" s="133"/>
+      <c r="B89" s="133"/>
+      <c r="C89" s="133"/>
       <c r="D89" s="30" t="s">
         <v>242</v>
       </c>
@@ -64303,9 +64303,9 @@
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A90" s="132"/>
-      <c r="B90" s="132"/>
-      <c r="C90" s="132"/>
+      <c r="A90" s="133"/>
+      <c r="B90" s="133"/>
+      <c r="C90" s="133"/>
       <c r="D90" s="30" t="s">
         <v>244</v>
       </c>
@@ -64314,9 +64314,9 @@
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A91" s="132"/>
-      <c r="B91" s="132"/>
-      <c r="C91" s="132"/>
+      <c r="A91" s="133"/>
+      <c r="B91" s="133"/>
+      <c r="C91" s="133"/>
       <c r="D91" s="30" t="s">
         <v>246</v>
       </c>
@@ -64325,16 +64325,16 @@
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A92" s="132"/>
-      <c r="B92" s="132"/>
-      <c r="C92" s="132"/>
+      <c r="A92" s="133"/>
+      <c r="B92" s="133"/>
+      <c r="C92" s="133"/>
       <c r="D92" s="28"/>
       <c r="E92" s="30"/>
     </row>
     <row r="93" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A93" s="132"/>
-      <c r="B93" s="136"/>
-      <c r="C93" s="132"/>
+      <c r="A93" s="133"/>
+      <c r="B93" s="138"/>
+      <c r="C93" s="133"/>
       <c r="D93" s="31" t="s">
         <v>248</v>
       </c>
@@ -64343,11 +64343,11 @@
       </c>
     </row>
     <row r="94" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="132" t="s">
+      <c r="A94" s="133" t="s">
         <v>156</v>
       </c>
-      <c r="B94" s="136"/>
-      <c r="C94" s="132" t="s">
+      <c r="B94" s="138"/>
+      <c r="C94" s="133" t="s">
         <v>109</v>
       </c>
       <c r="D94" s="28" t="s">
@@ -64358,9 +64358,9 @@
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A95" s="132"/>
-      <c r="B95" s="132"/>
-      <c r="C95" s="132"/>
+      <c r="A95" s="133"/>
+      <c r="B95" s="133"/>
+      <c r="C95" s="133"/>
       <c r="D95" s="28" t="s">
         <v>252</v>
       </c>
@@ -64369,9 +64369,9 @@
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A96" s="132"/>
-      <c r="B96" s="136"/>
-      <c r="C96" s="132"/>
+      <c r="A96" s="133"/>
+      <c r="B96" s="138"/>
+      <c r="C96" s="133"/>
       <c r="D96" s="31" t="s">
         <v>254</v>
       </c>
@@ -64383,7 +64383,7 @@
       <c r="A97" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B97" s="136" t="s">
+      <c r="B97" s="138" t="s">
         <v>84</v>
       </c>
       <c r="C97" s="31" t="s">
@@ -64397,11 +64397,11 @@
       </c>
     </row>
     <row r="98" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A98" s="132" t="s">
+      <c r="A98" s="133" t="s">
         <v>156</v>
       </c>
-      <c r="B98" s="136"/>
-      <c r="C98" s="132" t="s">
+      <c r="B98" s="138"/>
+      <c r="C98" s="133" t="s">
         <v>108</v>
       </c>
       <c r="D98" s="40" t="s">
@@ -64412,9 +64412,9 @@
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A99" s="132"/>
-      <c r="B99" s="132"/>
-      <c r="C99" s="132"/>
+      <c r="A99" s="133"/>
+      <c r="B99" s="133"/>
+      <c r="C99" s="133"/>
       <c r="D99" s="30" t="s">
         <v>242</v>
       </c>
@@ -64423,9 +64423,9 @@
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A100" s="132"/>
-      <c r="B100" s="132"/>
-      <c r="C100" s="132"/>
+      <c r="A100" s="133"/>
+      <c r="B100" s="133"/>
+      <c r="C100" s="133"/>
       <c r="D100" s="30" t="s">
         <v>244</v>
       </c>
@@ -64434,9 +64434,9 @@
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A101" s="132"/>
-      <c r="B101" s="132"/>
-      <c r="C101" s="132"/>
+      <c r="A101" s="133"/>
+      <c r="B101" s="133"/>
+      <c r="C101" s="133"/>
       <c r="D101" s="30" t="s">
         <v>246</v>
       </c>
@@ -64445,16 +64445,16 @@
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A102" s="132"/>
-      <c r="B102" s="132"/>
-      <c r="C102" s="132"/>
+      <c r="A102" s="133"/>
+      <c r="B102" s="133"/>
+      <c r="C102" s="133"/>
       <c r="D102" s="28"/>
       <c r="E102" s="30"/>
     </row>
     <row r="103" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A103" s="132"/>
-      <c r="B103" s="136"/>
-      <c r="C103" s="132"/>
+      <c r="A103" s="133"/>
+      <c r="B103" s="138"/>
+      <c r="C103" s="133"/>
       <c r="D103" s="31" t="s">
         <v>248</v>
       </c>
@@ -64463,11 +64463,11 @@
       </c>
     </row>
     <row r="104" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A104" s="132" t="s">
+      <c r="A104" s="133" t="s">
         <v>156</v>
       </c>
-      <c r="B104" s="136"/>
-      <c r="C104" s="132" t="s">
+      <c r="B104" s="138"/>
+      <c r="C104" s="133" t="s">
         <v>109</v>
       </c>
       <c r="D104" s="28" t="s">
@@ -64478,9 +64478,9 @@
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A105" s="132"/>
-      <c r="B105" s="132"/>
-      <c r="C105" s="132"/>
+      <c r="A105" s="133"/>
+      <c r="B105" s="133"/>
+      <c r="C105" s="133"/>
       <c r="D105" s="28" t="s">
         <v>252</v>
       </c>
@@ -64489,9 +64489,9 @@
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A106" s="132"/>
-      <c r="B106" s="136"/>
-      <c r="C106" s="132"/>
+      <c r="A106" s="133"/>
+      <c r="B106" s="138"/>
+      <c r="C106" s="133"/>
       <c r="D106" s="31" t="s">
         <v>254</v>
       </c>
@@ -64503,10 +64503,10 @@
       <c r="A107" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B107" s="132" t="s">
+      <c r="B107" s="133" t="s">
         <v>273</v>
       </c>
-      <c r="C107" s="132"/>
+      <c r="C107" s="133"/>
       <c r="D107" s="31" t="s">
         <v>274</v>
       </c>
@@ -64518,10 +64518,10 @@
       <c r="A108" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B108" s="132" t="s">
+      <c r="B108" s="133" t="s">
         <v>276</v>
       </c>
-      <c r="C108" s="132"/>
+      <c r="C108" s="133"/>
       <c r="D108" s="31" t="s">
         <v>277</v>
       </c>
@@ -64533,10 +64533,10 @@
       <c r="A109" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B109" s="132" t="s">
+      <c r="B109" s="133" t="s">
         <v>279</v>
       </c>
-      <c r="C109" s="132"/>
+      <c r="C109" s="133"/>
       <c r="D109" s="31" t="s">
         <v>280</v>
       </c>
@@ -64545,13 +64545,13 @@
       </c>
     </row>
     <row r="110" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="132" t="s">
+      <c r="A110" s="133" t="s">
         <v>156</v>
       </c>
-      <c r="B110" s="135" t="s">
+      <c r="B110" s="139" t="s">
         <v>51</v>
       </c>
-      <c r="C110" s="135"/>
+      <c r="C110" s="139"/>
       <c r="D110" s="39" t="s">
         <v>282</v>
       </c>
@@ -64560,16 +64560,16 @@
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A111" s="132"/>
-      <c r="B111" s="135"/>
-      <c r="C111" s="135"/>
+      <c r="A111" s="133"/>
+      <c r="B111" s="139"/>
+      <c r="C111" s="139"/>
       <c r="D111" s="41"/>
       <c r="E111" s="30"/>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A112" s="132"/>
-      <c r="B112" s="135"/>
-      <c r="C112" s="135"/>
+      <c r="A112" s="133"/>
+      <c r="B112" s="139"/>
+      <c r="C112" s="139"/>
       <c r="D112" s="42" t="s">
         <v>284</v>
       </c>
@@ -64578,9 +64578,9 @@
       </c>
     </row>
     <row r="113" spans="1:1024" x14ac:dyDescent="0.25">
-      <c r="A113" s="132"/>
-      <c r="B113" s="135"/>
-      <c r="C113" s="135"/>
+      <c r="A113" s="133"/>
+      <c r="B113" s="139"/>
+      <c r="C113" s="139"/>
       <c r="D113" s="42" t="s">
         <v>286</v>
       </c>
@@ -64589,9 +64589,9 @@
       </c>
     </row>
     <row r="114" spans="1:1024" x14ac:dyDescent="0.25">
-      <c r="A114" s="132"/>
-      <c r="B114" s="135"/>
-      <c r="C114" s="135"/>
+      <c r="A114" s="133"/>
+      <c r="B114" s="139"/>
+      <c r="C114" s="139"/>
       <c r="D114" s="42" t="s">
         <v>288</v>
       </c>
@@ -64600,9 +64600,9 @@
       </c>
     </row>
     <row r="115" spans="1:1024" x14ac:dyDescent="0.25">
-      <c r="A115" s="132"/>
-      <c r="B115" s="135"/>
-      <c r="C115" s="135"/>
+      <c r="A115" s="133"/>
+      <c r="B115" s="139"/>
+      <c r="C115" s="139"/>
       <c r="D115" s="43" t="s">
         <v>290</v>
       </c>
@@ -64648,10 +64648,10 @@
       <c r="A118" s="44" t="s">
         <v>179</v>
       </c>
-      <c r="B118" s="134" t="s">
+      <c r="B118" s="140" t="s">
         <v>62</v>
       </c>
-      <c r="C118" s="134"/>
+      <c r="C118" s="140"/>
       <c r="D118" s="46" t="s">
         <v>296</v>
       </c>
@@ -64912,10 +64912,10 @@
       <c r="IW118" s="44" t="s">
         <v>179</v>
       </c>
-      <c r="IX118" s="134" t="s">
+      <c r="IX118" s="140" t="s">
         <v>62</v>
       </c>
-      <c r="IY118" s="134"/>
+      <c r="IY118" s="140"/>
       <c r="IZ118" s="46" t="s">
         <v>296</v>
       </c>
@@ -65176,10 +65176,10 @@
       <c r="SS118" s="44" t="s">
         <v>179</v>
       </c>
-      <c r="ST118" s="134" t="s">
+      <c r="ST118" s="140" t="s">
         <v>62</v>
       </c>
-      <c r="SU118" s="134"/>
+      <c r="SU118" s="140"/>
       <c r="SV118" s="46" t="s">
         <v>296</v>
       </c>
@@ -65440,10 +65440,10 @@
       <c r="ACO118" s="44" t="s">
         <v>179</v>
       </c>
-      <c r="ACP118" s="134" t="s">
+      <c r="ACP118" s="140" t="s">
         <v>62</v>
       </c>
-      <c r="ACQ118" s="134"/>
+      <c r="ACQ118" s="140"/>
       <c r="ACR118" s="46" t="s">
         <v>296</v>
       </c>
@@ -65706,10 +65706,10 @@
       <c r="A119" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B119" s="132" t="s">
+      <c r="B119" s="133" t="s">
         <v>298</v>
       </c>
-      <c r="C119" s="132"/>
+      <c r="C119" s="133"/>
       <c r="D119" s="31" t="s">
         <v>299</v>
       </c>
@@ -65721,7 +65721,7 @@
       <c r="A120" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B120" s="132" t="s">
+      <c r="B120" s="133" t="s">
         <v>301</v>
       </c>
       <c r="C120" s="31" t="s">
@@ -65738,7 +65738,7 @@
       <c r="A121" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B121" s="132"/>
+      <c r="B121" s="133"/>
       <c r="C121" s="31" t="s">
         <v>102</v>
       </c>
@@ -65753,10 +65753,10 @@
       <c r="A122" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B122" s="132" t="s">
+      <c r="B122" s="133" t="s">
         <v>306</v>
       </c>
-      <c r="C122" s="132"/>
+      <c r="C122" s="133"/>
       <c r="D122" s="31" t="s">
         <v>307</v>
       </c>
@@ -65768,10 +65768,10 @@
       <c r="A123" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B123" s="132" t="s">
+      <c r="B123" s="133" t="s">
         <v>72</v>
       </c>
-      <c r="C123" s="132"/>
+      <c r="C123" s="133"/>
       <c r="D123" s="31" t="s">
         <v>309</v>
       </c>
@@ -65783,10 +65783,10 @@
       <c r="A124" s="27" t="s">
         <v>156</v>
       </c>
-      <c r="B124" s="133" t="s">
+      <c r="B124" s="134" t="s">
         <v>57</v>
       </c>
-      <c r="C124" s="133"/>
+      <c r="C124" s="134"/>
       <c r="D124" s="27" t="s">
         <v>311</v>
       </c>
@@ -65798,10 +65798,10 @@
       <c r="A125" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B125" s="132" t="s">
+      <c r="B125" s="133" t="s">
         <v>56</v>
       </c>
-      <c r="C125" s="132"/>
+      <c r="C125" s="133"/>
       <c r="D125" s="27" t="s">
         <v>313</v>
       </c>
@@ -65813,10 +65813,10 @@
       <c r="A126" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B126" s="132" t="s">
+      <c r="B126" s="133" t="s">
         <v>54</v>
       </c>
-      <c r="C126" s="132"/>
+      <c r="C126" s="133"/>
       <c r="D126" s="27" t="s">
         <v>315</v>
       </c>
@@ -65828,10 +65828,10 @@
       <c r="A127" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B127" s="132" t="s">
+      <c r="B127" s="133" t="s">
         <v>55</v>
       </c>
-      <c r="C127" s="132"/>
+      <c r="C127" s="133"/>
       <c r="D127" s="27" t="s">
         <v>317</v>
       </c>
@@ -65840,13 +65840,13 @@
       </c>
     </row>
     <row r="128" spans="1:1024" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A128" s="132" t="s">
+      <c r="A128" s="133" t="s">
         <v>156</v>
       </c>
-      <c r="B128" s="132" t="s">
+      <c r="B128" s="133" t="s">
         <v>53</v>
       </c>
-      <c r="C128" s="132"/>
+      <c r="C128" s="133"/>
       <c r="D128" s="28" t="s">
         <v>319</v>
       </c>
@@ -65855,16 +65855,16 @@
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A129" s="132"/>
-      <c r="B129" s="132"/>
-      <c r="C129" s="132"/>
+      <c r="A129" s="133"/>
+      <c r="B129" s="133"/>
+      <c r="C129" s="133"/>
       <c r="D129" s="28"/>
       <c r="E129" s="30"/>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A130" s="132"/>
-      <c r="B130" s="132"/>
-      <c r="C130" s="132"/>
+      <c r="A130" s="133"/>
+      <c r="B130" s="133"/>
+      <c r="C130" s="133"/>
       <c r="D130" s="28" t="s">
         <v>321</v>
       </c>
@@ -65873,9 +65873,9 @@
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A131" s="132"/>
-      <c r="B131" s="132"/>
-      <c r="C131" s="132"/>
+      <c r="A131" s="133"/>
+      <c r="B131" s="133"/>
+      <c r="C131" s="133"/>
       <c r="D131" s="28" t="s">
         <v>323</v>
       </c>
@@ -65884,9 +65884,9 @@
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A132" s="132"/>
-      <c r="B132" s="132"/>
-      <c r="C132" s="132"/>
+      <c r="A132" s="133"/>
+      <c r="B132" s="133"/>
+      <c r="C132" s="133"/>
       <c r="D132" s="28" t="s">
         <v>325</v>
       </c>
@@ -65895,9 +65895,9 @@
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A133" s="132"/>
-      <c r="B133" s="132"/>
-      <c r="C133" s="132"/>
+      <c r="A133" s="133"/>
+      <c r="B133" s="133"/>
+      <c r="C133" s="133"/>
       <c r="D133" s="31" t="s">
         <v>327</v>
       </c>
@@ -65909,10 +65909,10 @@
       <c r="A134" s="32" t="s">
         <v>179</v>
       </c>
-      <c r="B134" s="132" t="s">
+      <c r="B134" s="133" t="s">
         <v>89</v>
       </c>
-      <c r="C134" s="132"/>
+      <c r="C134" s="133"/>
       <c r="D134" s="31" t="s">
         <v>329</v>
       </c>
@@ -65924,10 +65924,10 @@
       <c r="A135" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B135" s="132" t="s">
+      <c r="B135" s="133" t="s">
         <v>66</v>
       </c>
-      <c r="C135" s="132"/>
+      <c r="C135" s="133"/>
       <c r="D135" s="31" t="s">
         <v>331</v>
       </c>
@@ -65939,10 +65939,10 @@
       <c r="A136" s="32" t="s">
         <v>156</v>
       </c>
-      <c r="B136" s="132" t="s">
+      <c r="B136" s="133" t="s">
         <v>333</v>
       </c>
-      <c r="C136" s="132"/>
+      <c r="C136" s="133"/>
       <c r="D136" s="31" t="s">
         <v>334</v>
       </c>
@@ -65954,10 +65954,10 @@
       <c r="A137" s="32" t="s">
         <v>179</v>
       </c>
-      <c r="B137" s="132" t="s">
+      <c r="B137" s="133" t="s">
         <v>88</v>
       </c>
-      <c r="C137" s="132"/>
+      <c r="C137" s="133"/>
       <c r="D137" s="31" t="s">
         <v>336</v>
       </c>
@@ -65969,10 +65969,10 @@
       <c r="A138" s="32" t="s">
         <v>179</v>
       </c>
-      <c r="B138" s="132" t="s">
+      <c r="B138" s="133" t="s">
         <v>58</v>
       </c>
-      <c r="C138" s="132"/>
+      <c r="C138" s="133"/>
       <c r="D138" s="31" t="s">
         <v>338</v>
       </c>
@@ -65981,12 +65981,12 @@
       </c>
     </row>
     <row r="140" spans="1:5" ht="118.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A140" s="133" t="s">
+      <c r="A140" s="134" t="s">
         <v>340</v>
       </c>
-      <c r="B140" s="133"/>
-      <c r="C140" s="133"/>
-      <c r="D140" s="133"/>
+      <c r="B140" s="134"/>
+      <c r="C140" s="134"/>
+      <c r="D140" s="134"/>
       <c r="E140" s="27" t="s">
         <v>341</v>
       </c>
@@ -65998,21 +65998,55 @@
     </row>
   </sheetData>
   <mergeCells count="72">
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="A5:A11"/>
-    <mergeCell ref="B5:C11"/>
-    <mergeCell ref="B12:B16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="A23:A36"/>
-    <mergeCell ref="B23:C36"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B135:C135"/>
+    <mergeCell ref="B136:C136"/>
+    <mergeCell ref="B137:C137"/>
+    <mergeCell ref="B138:C138"/>
+    <mergeCell ref="A140:D140"/>
+    <mergeCell ref="B126:C126"/>
+    <mergeCell ref="B127:C127"/>
+    <mergeCell ref="A128:A133"/>
+    <mergeCell ref="B128:C133"/>
+    <mergeCell ref="B134:C134"/>
+    <mergeCell ref="B120:B121"/>
+    <mergeCell ref="B122:C122"/>
+    <mergeCell ref="B123:C123"/>
+    <mergeCell ref="B124:C124"/>
+    <mergeCell ref="B125:C125"/>
+    <mergeCell ref="B118:C118"/>
+    <mergeCell ref="IX118:IY118"/>
+    <mergeCell ref="ST118:SU118"/>
+    <mergeCell ref="ACP118:ACQ118"/>
+    <mergeCell ref="B119:C119"/>
+    <mergeCell ref="B107:C107"/>
+    <mergeCell ref="B108:C108"/>
+    <mergeCell ref="B109:C109"/>
+    <mergeCell ref="A110:A115"/>
+    <mergeCell ref="B110:C115"/>
+    <mergeCell ref="B97:B106"/>
+    <mergeCell ref="A98:A103"/>
+    <mergeCell ref="C98:C103"/>
+    <mergeCell ref="A104:A106"/>
+    <mergeCell ref="C104:C106"/>
+    <mergeCell ref="A80:A85"/>
+    <mergeCell ref="B80:C85"/>
+    <mergeCell ref="B86:C86"/>
+    <mergeCell ref="B87:B96"/>
+    <mergeCell ref="A88:A93"/>
+    <mergeCell ref="C88:C93"/>
+    <mergeCell ref="A94:A96"/>
+    <mergeCell ref="C94:C96"/>
+    <mergeCell ref="B70:B79"/>
+    <mergeCell ref="A71:A76"/>
+    <mergeCell ref="C71:C76"/>
+    <mergeCell ref="A77:A79"/>
+    <mergeCell ref="C77:C79"/>
+    <mergeCell ref="B59:C59"/>
+    <mergeCell ref="B60:B69"/>
+    <mergeCell ref="A61:A66"/>
+    <mergeCell ref="C61:C66"/>
+    <mergeCell ref="A67:A69"/>
+    <mergeCell ref="C67:C69"/>
     <mergeCell ref="A40:A44"/>
     <mergeCell ref="B40:C44"/>
     <mergeCell ref="B45:C45"/>
@@ -66021,55 +66055,21 @@
     <mergeCell ref="C50:C55"/>
     <mergeCell ref="A56:A58"/>
     <mergeCell ref="C56:C58"/>
-    <mergeCell ref="B59:C59"/>
-    <mergeCell ref="B60:B69"/>
-    <mergeCell ref="A61:A66"/>
-    <mergeCell ref="C61:C66"/>
-    <mergeCell ref="A67:A69"/>
-    <mergeCell ref="C67:C69"/>
-    <mergeCell ref="B70:B79"/>
-    <mergeCell ref="A71:A76"/>
-    <mergeCell ref="C71:C76"/>
-    <mergeCell ref="A77:A79"/>
-    <mergeCell ref="C77:C79"/>
-    <mergeCell ref="A80:A85"/>
-    <mergeCell ref="B80:C85"/>
-    <mergeCell ref="B86:C86"/>
-    <mergeCell ref="B87:B96"/>
-    <mergeCell ref="A88:A93"/>
-    <mergeCell ref="C88:C93"/>
-    <mergeCell ref="A94:A96"/>
-    <mergeCell ref="C94:C96"/>
-    <mergeCell ref="B97:B106"/>
-    <mergeCell ref="A98:A103"/>
-    <mergeCell ref="C98:C103"/>
-    <mergeCell ref="A104:A106"/>
-    <mergeCell ref="C104:C106"/>
-    <mergeCell ref="B107:C107"/>
-    <mergeCell ref="B108:C108"/>
-    <mergeCell ref="B109:C109"/>
-    <mergeCell ref="A110:A115"/>
-    <mergeCell ref="B110:C115"/>
-    <mergeCell ref="B118:C118"/>
-    <mergeCell ref="IX118:IY118"/>
-    <mergeCell ref="ST118:SU118"/>
-    <mergeCell ref="ACP118:ACQ118"/>
-    <mergeCell ref="B119:C119"/>
-    <mergeCell ref="B120:B121"/>
-    <mergeCell ref="B122:C122"/>
-    <mergeCell ref="B123:C123"/>
-    <mergeCell ref="B124:C124"/>
-    <mergeCell ref="B125:C125"/>
-    <mergeCell ref="B126:C126"/>
-    <mergeCell ref="B127:C127"/>
-    <mergeCell ref="A128:A133"/>
-    <mergeCell ref="B128:C133"/>
-    <mergeCell ref="B134:C134"/>
-    <mergeCell ref="B135:C135"/>
-    <mergeCell ref="B136:C136"/>
-    <mergeCell ref="B137:C137"/>
-    <mergeCell ref="B138:C138"/>
-    <mergeCell ref="A140:D140"/>
+    <mergeCell ref="A23:A36"/>
+    <mergeCell ref="B23:C36"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="A5:A11"/>
+    <mergeCell ref="B5:C11"/>
+    <mergeCell ref="B12:B16"/>
+    <mergeCell ref="B17:C17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="8" fitToHeight="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>